<commit_message>
Actualizar formularios y gestión MIPE
</commit_message>
<xml_diff>
--- a/assets/ASEGURAMIENTO DE PLAGUICIDAS A LA LLEGADA AL ALMACEN.xlsx
+++ b/assets/ASEGURAMIENTO DE PLAGUICIDAS A LA LLEGADA AL ALMACEN.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Nueva carpeta\flutter_application_1\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Nueva carpeta\flutter_application_1 - android - copia\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C013ADE1-4623-4E4F-8B51-4CE9DF3524BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B7A3BD0-A67D-4E0D-936C-A63CD20D0F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{42B04D72-A3C2-464D-95D4-0C30DAB9C8E5}"/>
   </bookViews>
@@ -30,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -42,18 +40,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>CULTIVOS LA PLANICIE S.A.S.</t>
   </si>
   <si>
-    <t>Versión 1</t>
-  </si>
-  <si>
     <t>MIPE</t>
-  </si>
-  <si>
-    <t>Diciembre 2020</t>
   </si>
   <si>
     <t>ASEGURAMIENTO DE PLAGUICIDAS A LA LLEGADA AL ALMACEN</t>
@@ -129,7 +121,10 @@
     <t>DENSIDAD</t>
   </si>
   <si>
-    <t>(CANTIDAD)</t>
+    <t>Versión 2</t>
+  </si>
+  <si>
+    <t>Septiembre 2026</t>
   </si>
 </sst>
 </file>
@@ -203,7 +198,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -381,6 +376,19 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -400,12 +408,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -500,6 +502,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2239,81 +2247,81 @@
   <sheetData>
     <row r="1" spans="2:21" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="39" t="s">
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
-      <c r="N2" s="39"/>
-      <c r="O2" s="39"/>
-      <c r="P2" s="39"/>
-      <c r="Q2" s="39"/>
-      <c r="R2" s="39"/>
-      <c r="S2" s="39"/>
-      <c r="T2" s="39"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
       <c r="U2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="38" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="40" t="s">
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="38"/>
+      <c r="U3" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="3" t="s">
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="41" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
-      <c r="L4" s="41"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="41"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="41"/>
-      <c r="Q4" s="41"/>
-      <c r="R4" s="41"/>
-      <c r="S4" s="41"/>
-      <c r="T4" s="41"/>
-      <c r="U4" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="5" spans="2:21" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -2324,679 +2332,677 @@
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
     </row>
-    <row r="6" spans="2:21" s="35" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="36"/>
-      <c r="J6" s="42" t="s">
+    <row r="6" spans="2:21" s="33" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="34"/>
+      <c r="J6" s="40" t="s">
+        <v>4</v>
+      </c>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="40" t="s">
+        <v>5</v>
+      </c>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="42"/>
+      <c r="R6" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="44"/>
-      <c r="N6" s="42" t="s">
+      <c r="S6" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="O6" s="43"/>
-      <c r="P6" s="43"/>
-      <c r="Q6" s="44"/>
-      <c r="R6" s="45" t="s">
+      <c r="T6" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="S6" s="47" t="s">
+      <c r="U6" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="T6" s="49" t="s">
+    </row>
+    <row r="7" spans="2:21" s="35" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="U6" s="52" t="s">
+      <c r="C7" s="47" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="2:21" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="54" t="s">
+      <c r="D7" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="E7" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="F7" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="G7" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="H7" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="49" t="s">
+      <c r="I7" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="47" t="s">
+      <c r="J7" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="52" t="s">
+      <c r="K7" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="46" t="s">
+      <c r="L7" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="50" t="s">
+      <c r="M7" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="N7" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="53" t="s">
+      <c r="O7" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="N7" s="46" t="s">
+      <c r="P7" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="O7" s="48" t="s">
+      <c r="Q7" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="P7" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q7" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="46"/>
-      <c r="S7" s="48"/>
-      <c r="T7" s="50"/>
+      <c r="R7" s="44"/>
+      <c r="S7" s="46"/>
+      <c r="T7" s="48"/>
       <c r="U7" s="53"/>
     </row>
-    <row r="8" spans="2:21" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" s="35" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="55"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" s="50"/>
-      <c r="H8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="46"/>
       <c r="I8" s="53"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="48"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="46"/>
       <c r="M8" s="53"/>
       <c r="N8" s="55"/>
-      <c r="O8" s="48"/>
-      <c r="P8" s="48"/>
+      <c r="O8" s="46"/>
+      <c r="P8" s="46"/>
       <c r="Q8" s="56"/>
-      <c r="R8" s="46"/>
-      <c r="S8" s="48"/>
-      <c r="T8" s="50"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="46"/>
+      <c r="T8" s="48"/>
       <c r="U8" s="53"/>
     </row>
     <row r="9" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="15"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="18"/>
-      <c r="U9" s="19"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="16"/>
+      <c r="U9" s="17"/>
     </row>
     <row r="10" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="20"/>
-      <c r="T10" s="18"/>
-      <c r="U10" s="19"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="14"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="17"/>
     </row>
     <row r="11" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="8"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="16"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="18"/>
-      <c r="U11" s="19"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="14"/>
+      <c r="S11" s="18"/>
+      <c r="T11" s="16"/>
+      <c r="U11" s="17"/>
     </row>
     <row r="12" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="16"/>
-      <c r="S12" s="20"/>
-      <c r="T12" s="18"/>
-      <c r="U12" s="19"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="14"/>
+      <c r="S12" s="18"/>
+      <c r="T12" s="16"/>
+      <c r="U12" s="17"/>
     </row>
     <row r="13" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="8"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="22"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="19"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="21"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="21"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9"/>
+      <c r="U13" s="19"/>
     </row>
     <row r="14" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="8"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="19"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="21"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="20"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="21"/>
+      <c r="S14" s="9"/>
+      <c r="T14" s="9"/>
+      <c r="U14" s="19"/>
     </row>
     <row r="15" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="8"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="23"/>
-      <c r="S15" s="11"/>
-      <c r="T15" s="11"/>
-      <c r="U15" s="21"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="21"/>
+      <c r="S15" s="9"/>
+      <c r="T15" s="9"/>
+      <c r="U15" s="19"/>
     </row>
     <row r="16" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="8"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="18"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-      <c r="U16" s="21"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="21"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9"/>
+      <c r="U16" s="19"/>
     </row>
     <row r="17" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="8"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="18"/>
-      <c r="P17" s="18"/>
-      <c r="Q17" s="19"/>
-      <c r="R17" s="23"/>
-      <c r="S17" s="11"/>
-      <c r="T17" s="11"/>
-      <c r="U17" s="21"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="21"/>
+      <c r="S17" s="9"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="19"/>
     </row>
     <row r="18" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="8"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="18"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="19"/>
-      <c r="R18" s="23"/>
-      <c r="S18" s="11"/>
-      <c r="T18" s="11"/>
-      <c r="U18" s="21"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="9"/>
+      <c r="T18" s="9"/>
+      <c r="U18" s="19"/>
     </row>
     <row r="19" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="8"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="19"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="11"/>
-      <c r="T19" s="11"/>
-      <c r="U19" s="21"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="9"/>
+      <c r="U19" s="19"/>
     </row>
     <row r="20" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="8"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="18"/>
-      <c r="P20" s="18"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="23"/>
-      <c r="S20" s="11"/>
-      <c r="T20" s="11"/>
-      <c r="U20" s="21"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="9"/>
+      <c r="T20" s="9"/>
+      <c r="U20" s="19"/>
     </row>
     <row r="21" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="8"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="18"/>
-      <c r="P21" s="18"/>
-      <c r="Q21" s="19"/>
-      <c r="R21" s="23"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="21"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="21"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="19"/>
     </row>
     <row r="22" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="8"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="18"/>
-      <c r="Q22" s="19"/>
-      <c r="R22" s="23"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="21"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="20"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="9"/>
+      <c r="T22" s="9"/>
+      <c r="U22" s="19"/>
     </row>
     <row r="23" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="8"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="18"/>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="11"/>
-      <c r="T23" s="11"/>
-      <c r="U23" s="21"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="9"/>
+      <c r="T23" s="9"/>
+      <c r="U23" s="19"/>
     </row>
     <row r="24" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="8"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="22"/>
-      <c r="O24" s="18"/>
-      <c r="P24" s="18"/>
-      <c r="Q24" s="19"/>
-      <c r="R24" s="23"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-      <c r="U24" s="21"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="21"/>
+      <c r="S24" s="9"/>
+      <c r="T24" s="9"/>
+      <c r="U24" s="19"/>
     </row>
     <row r="25" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="8"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="18"/>
-      <c r="Q25" s="19"/>
-      <c r="R25" s="23"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="21"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="21"/>
+      <c r="S25" s="9"/>
+      <c r="T25" s="9"/>
+      <c r="U25" s="19"/>
     </row>
     <row r="26" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="8"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="22"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="22"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="18"/>
-      <c r="Q26" s="19"/>
-      <c r="R26" s="23"/>
-      <c r="S26" s="11"/>
-      <c r="T26" s="11"/>
-      <c r="U26" s="21"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="20"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="21"/>
+      <c r="S26" s="9"/>
+      <c r="T26" s="9"/>
+      <c r="U26" s="19"/>
     </row>
     <row r="27" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="8"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="18"/>
-      <c r="L27" s="18"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="18"/>
-      <c r="P27" s="18"/>
-      <c r="Q27" s="19"/>
-      <c r="R27" s="23"/>
-      <c r="S27" s="11"/>
-      <c r="T27" s="11"/>
-      <c r="U27" s="21"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="20"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="21"/>
+      <c r="S27" s="9"/>
+      <c r="T27" s="9"/>
+      <c r="U27" s="19"/>
     </row>
     <row r="28" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="8"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="22"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="19"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="11"/>
-      <c r="T28" s="11"/>
-      <c r="U28" s="21"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="17"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="17"/>
+      <c r="R28" s="21"/>
+      <c r="S28" s="9"/>
+      <c r="T28" s="9"/>
+      <c r="U28" s="19"/>
     </row>
     <row r="29" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="8"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="18"/>
-      <c r="P29" s="18"/>
-      <c r="Q29" s="19"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="11"/>
-      <c r="T29" s="11"/>
-      <c r="U29" s="21"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="20"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="17"/>
+      <c r="R29" s="21"/>
+      <c r="S29" s="9"/>
+      <c r="T29" s="9"/>
+      <c r="U29" s="19"/>
     </row>
     <row r="30" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="8"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="18"/>
-      <c r="L30" s="18"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="22"/>
-      <c r="O30" s="18"/>
-      <c r="P30" s="18"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="23"/>
-      <c r="S30" s="11"/>
-      <c r="T30" s="11"/>
-      <c r="U30" s="21"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="20"/>
+      <c r="O30" s="16"/>
+      <c r="P30" s="16"/>
+      <c r="Q30" s="17"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="9"/>
+      <c r="U30" s="19"/>
     </row>
     <row r="31" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="8"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="22"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="19"/>
-      <c r="N31" s="22"/>
-      <c r="O31" s="18"/>
-      <c r="P31" s="18"/>
-      <c r="Q31" s="19"/>
-      <c r="R31" s="23"/>
-      <c r="S31" s="11"/>
-      <c r="T31" s="11"/>
-      <c r="U31" s="21"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="17"/>
+      <c r="N31" s="20"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="17"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="9"/>
+      <c r="T31" s="9"/>
+      <c r="U31" s="19"/>
     </row>
     <row r="32" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="8"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="22"/>
-      <c r="O32" s="18"/>
-      <c r="P32" s="18"/>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="11"/>
-      <c r="T32" s="11"/>
-      <c r="U32" s="21"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
+      <c r="M32" s="17"/>
+      <c r="N32" s="20"/>
+      <c r="O32" s="16"/>
+      <c r="P32" s="16"/>
+      <c r="Q32" s="17"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="9"/>
+      <c r="T32" s="9"/>
+      <c r="U32" s="19"/>
     </row>
     <row r="33" spans="2:21" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="24"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="28"/>
-      <c r="L33" s="28"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="27"/>
-      <c r="O33" s="28"/>
-      <c r="P33" s="28"/>
-      <c r="Q33" s="29"/>
-      <c r="R33" s="30"/>
-      <c r="S33" s="25"/>
-      <c r="T33" s="25"/>
-      <c r="U33" s="26"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="27"/>
+      <c r="N33" s="25"/>
+      <c r="O33" s="26"/>
+      <c r="P33" s="26"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="28"/>
+      <c r="S33" s="23"/>
+      <c r="T33" s="23"/>
+      <c r="U33" s="24"/>
     </row>
     <row r="34" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="R34" s="31"/>
+      <c r="R34" s="29"/>
     </row>
     <row r="35" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="32"/>
-      <c r="K35" s="32"/>
-      <c r="L35" s="32"/>
-      <c r="M35" s="32"/>
-      <c r="N35" s="32"/>
-      <c r="O35" s="32"/>
-      <c r="R35" s="31"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="30"/>
+      <c r="M35" s="30"/>
+      <c r="N35" s="30"/>
+      <c r="O35" s="30"/>
+      <c r="R35" s="29"/>
     </row>
     <row r="36" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F36" s="32"/>
+      <c r="F36" s="30"/>
       <c r="G36" s="51"/>
       <c r="H36" s="51"/>
       <c r="I36" s="51"/>
@@ -3004,147 +3010,147 @@
       <c r="K36" s="51"/>
       <c r="L36" s="51"/>
       <c r="M36" s="51"/>
-      <c r="N36" s="33"/>
-      <c r="O36" s="33"/>
-      <c r="R36" s="31"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="31"/>
+      <c r="R36" s="29"/>
     </row>
     <row r="37" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="32"/>
-      <c r="K37" s="32"/>
-      <c r="L37" s="32"/>
-      <c r="M37" s="32"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="32"/>
+      <c r="O37" s="32"/>
       <c r="P37" s="5"/>
       <c r="Q37" s="5"/>
       <c r="R37" s="5"/>
     </row>
     <row r="38" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="32"/>
-      <c r="J38" s="33"/>
-      <c r="K38" s="33"/>
-      <c r="L38" s="33"/>
-      <c r="M38" s="33"/>
-      <c r="N38" s="33"/>
-      <c r="O38" s="33"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="31"/>
+      <c r="K38" s="31"/>
+      <c r="L38" s="31"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="31"/>
     </row>
     <row r="39" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="33"/>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
-      <c r="M39" s="33"/>
-      <c r="N39" s="33"/>
-      <c r="O39" s="33"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="30"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="31"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="31"/>
     </row>
     <row r="40" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="32"/>
-      <c r="J40" s="33"/>
-      <c r="K40" s="33"/>
-      <c r="L40" s="33"/>
-      <c r="M40" s="33"/>
-      <c r="N40" s="33"/>
-      <c r="O40" s="33"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="30"/>
+      <c r="I40" s="30"/>
+      <c r="J40" s="31"/>
+      <c r="K40" s="31"/>
+      <c r="L40" s="31"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="31"/>
+      <c r="O40" s="31"/>
     </row>
     <row r="41" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="32"/>
-      <c r="J41" s="33"/>
-      <c r="K41" s="33"/>
-      <c r="L41" s="33"/>
-      <c r="M41" s="33"/>
-      <c r="N41" s="33"/>
-      <c r="O41" s="33"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="30"/>
+      <c r="H41" s="30"/>
+      <c r="I41" s="30"/>
+      <c r="J41" s="31"/>
+      <c r="K41" s="31"/>
+      <c r="L41" s="31"/>
+      <c r="M41" s="31"/>
+      <c r="N41" s="31"/>
+      <c r="O41" s="31"/>
     </row>
     <row r="42" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
-      <c r="M42" s="33"/>
-      <c r="N42" s="33"/>
-      <c r="O42" s="33"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30"/>
+      <c r="H42" s="30"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+      <c r="L42" s="31"/>
+      <c r="M42" s="31"/>
+      <c r="N42" s="31"/>
+      <c r="O42" s="31"/>
     </row>
     <row r="43" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
-      <c r="J43" s="33"/>
-      <c r="K43" s="33"/>
-      <c r="L43" s="33"/>
-      <c r="M43" s="33"/>
-      <c r="N43" s="33"/>
-      <c r="O43" s="33"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="30"/>
+      <c r="J43" s="31"/>
+      <c r="K43" s="31"/>
+      <c r="L43" s="31"/>
+      <c r="M43" s="31"/>
+      <c r="N43" s="31"/>
+      <c r="O43" s="31"/>
     </row>
     <row r="44" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="32"/>
-      <c r="J44" s="33"/>
-      <c r="K44" s="33"/>
-      <c r="L44" s="33"/>
-      <c r="M44" s="33"/>
-      <c r="N44" s="33"/>
-      <c r="O44" s="33"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="30"/>
+      <c r="I44" s="30"/>
+      <c r="J44" s="31"/>
+      <c r="K44" s="31"/>
+      <c r="L44" s="31"/>
+      <c r="M44" s="31"/>
+      <c r="N44" s="31"/>
+      <c r="O44" s="31"/>
     </row>
     <row r="45" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="32"/>
-      <c r="J45" s="33"/>
-      <c r="K45" s="33"/>
-      <c r="L45" s="33"/>
-      <c r="M45" s="33"/>
-      <c r="N45" s="33"/>
-      <c r="O45" s="33"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
+      <c r="J45" s="31"/>
+      <c r="K45" s="31"/>
+      <c r="L45" s="31"/>
+      <c r="M45" s="31"/>
+      <c r="N45" s="31"/>
+      <c r="O45" s="31"/>
     </row>
     <row r="46" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
-      <c r="H46" s="32"/>
-      <c r="I46" s="32"/>
-      <c r="J46" s="33"/>
-      <c r="K46" s="33"/>
-      <c r="L46" s="33"/>
-      <c r="M46" s="33"/>
-      <c r="N46" s="33"/>
-      <c r="O46" s="33"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="31"/>
+      <c r="K46" s="31"/>
+      <c r="L46" s="31"/>
+      <c r="M46" s="31"/>
+      <c r="N46" s="31"/>
+      <c r="O46" s="31"/>
     </row>
     <row r="47" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="32"/>
-      <c r="J47" s="33"/>
-      <c r="K47" s="33"/>
-      <c r="L47" s="33"/>
-      <c r="M47" s="33"/>
-      <c r="N47" s="33"/>
-      <c r="O47" s="33"/>
+      <c r="F47" s="30"/>
+      <c r="G47" s="30"/>
+      <c r="H47" s="30"/>
+      <c r="I47" s="30"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="31"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="G36:M36"/>
     <mergeCell ref="U6:U8"/>
     <mergeCell ref="B7:B8"/>
@@ -3171,10 +3177,11 @@
     <mergeCell ref="S6:S8"/>
     <mergeCell ref="T6:T8"/>
     <mergeCell ref="L7:L8"/>
+    <mergeCell ref="F7:F8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="51" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="49" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>

</xml_diff>